<commit_message>
Debug until feasible result returned
Debug until feasible result returned
</commit_message>
<xml_diff>
--- a/test/production/staff_requested_duty_excel.xlsx
+++ b/test/production/staff_requested_duty_excel.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>C(1)</t>
   </si>
@@ -103,6 +103,9 @@
   </si>
   <si>
     <t>X(1)</t>
+  </si>
+  <si>
+    <t>X(2)</t>
   </si>
   <si>
     <t>LYG(1)</t>
@@ -253,12 +256,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -867,7 +871,9 @@
       <c r="AD1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="AE1" s="3"/>
+      <c r="AE1" s="5" t="s">
+        <v>29</v>
+      </c>
       <c r="AF1" s="3"/>
       <c r="AG1" s="3"/>
       <c r="AH1" s="3"/>
@@ -876,14 +882,14 @@
     </row>
     <row r="2" ht="14.25">
       <c r="A2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="5" t="s">
-        <v>30</v>
+      <c r="G2" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="H2" s="1"/>
       <c r="I2"/>
@@ -895,26 +901,26 @@
       <c r="O2" s="1"/>
       <c r="P2"/>
       <c r="Q2"/>
-      <c r="R2" s="6"/>
+      <c r="R2" s="7"/>
       <c r="S2" s="2"/>
       <c r="T2" s="2"/>
-      <c r="U2" s="6"/>
+      <c r="U2" s="7"/>
       <c r="V2" s="1"/>
       <c r="W2"/>
       <c r="X2"/>
       <c r="Y2"/>
       <c r="Z2" s="2"/>
       <c r="AA2" s="2"/>
-      <c r="AB2" s="6"/>
+      <c r="AB2" s="7"/>
       <c r="AC2" s="1"/>
       <c r="AD2" s="2"/>
     </row>
     <row r="3" ht="14.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="6"/>
+      <c r="D3" s="7"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3"/>
@@ -931,35 +937,35 @@
       <c r="R3"/>
       <c r="S3" s="2"/>
       <c r="T3" s="2"/>
-      <c r="U3" s="6"/>
+      <c r="U3" s="7"/>
       <c r="V3" s="1"/>
       <c r="W3"/>
       <c r="X3"/>
       <c r="Y3"/>
       <c r="Z3" s="2"/>
-      <c r="AA3" s="5" t="s">
-        <v>32</v>
+      <c r="AA3" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="AB3"/>
-      <c r="AC3" s="7" t="s">
-        <v>30</v>
+      <c r="AC3" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="AD3" s="2"/>
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C4" s="2"/>
-      <c r="D4" s="6"/>
+      <c r="D4" s="7"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4"/>
       <c r="H4" s="1"/>
       <c r="I4"/>
       <c r="J4"/>
-      <c r="K4" s="5" t="s">
-        <v>32</v>
+      <c r="K4" s="6" t="s">
+        <v>33</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
@@ -976,29 +982,29 @@
       <c r="X4"/>
       <c r="Y4"/>
       <c r="Z4" s="2"/>
-      <c r="AA4" s="6"/>
+      <c r="AA4" s="7"/>
       <c r="AB4"/>
       <c r="AC4" s="1"/>
       <c r="AD4" s="2"/>
     </row>
     <row r="5" s="3" customFormat="1" ht="14.25">
       <c r="A5" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>30</v>
+        <v>35</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
-      <c r="F5" s="9"/>
+      <c r="F5" s="10"/>
       <c r="G5" s="3"/>
       <c r="H5" s="4"/>
       <c r="I5" s="3"/>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
-      <c r="L5" s="8" t="s">
-        <v>32</v>
+      <c r="L5" s="9" t="s">
+        <v>33</v>
       </c>
       <c r="M5" s="3"/>
       <c r="N5" s="3"/>
@@ -1013,7 +1019,7 @@
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
       <c r="Y5" s="3"/>
-      <c r="Z5" s="9"/>
+      <c r="Z5" s="10"/>
       <c r="AA5" s="3"/>
       <c r="AB5" s="3"/>
       <c r="AC5" s="4"/>
@@ -1029,12 +1035,12 @@
     </row>
     <row r="6" ht="14.25">
       <c r="A6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="5" t="s">
-        <v>30</v>
+        <v>36</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6"/>
@@ -1054,8 +1060,8 @@
       <c r="U6"/>
       <c r="V6" s="1"/>
       <c r="W6"/>
-      <c r="X6" s="5" t="s">
-        <v>30</v>
+      <c r="X6" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="Y6"/>
       <c r="Z6" s="2"/>
@@ -1066,7 +1072,7 @@
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -1087,19 +1093,19 @@
       <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7"/>
-      <c r="V7" s="10"/>
+      <c r="V7" s="11"/>
       <c r="W7"/>
       <c r="X7"/>
       <c r="Y7"/>
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
       <c r="AB7"/>
-      <c r="AC7" s="10"/>
+      <c r="AC7" s="11"/>
       <c r="AD7" s="2"/>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -1110,16 +1116,16 @@
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
-      <c r="L8" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>30</v>
+      <c r="L8" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="N8"/>
       <c r="O8" s="1"/>
       <c r="P8"/>
-      <c r="Q8" s="6"/>
+      <c r="Q8" s="7"/>
       <c r="R8"/>
       <c r="S8" s="2"/>
       <c r="T8" s="2"/>
@@ -1130,24 +1136,24 @@
       <c r="Y8"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
-      <c r="AB8" s="6"/>
+      <c r="AB8" s="7"/>
       <c r="AC8" s="1"/>
       <c r="AD8" s="2"/>
     </row>
     <row r="9" s="3" customFormat="1" ht="14.25">
       <c r="A9" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="C9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>30</v>
+      <c r="C9" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>31</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="9"/>
+      <c r="G9" s="10"/>
       <c r="H9" s="4"/>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -1166,7 +1172,7 @@
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
       <c r="Y9" s="3"/>
-      <c r="Z9" s="9"/>
+      <c r="Z9" s="10"/>
       <c r="AA9" s="3"/>
       <c r="AB9" s="3"/>
       <c r="AC9" s="4"/>
@@ -1183,14 +1189,14 @@
     </row>
     <row r="10" ht="14.25">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
       <c r="G10"/>
-      <c r="H10" s="10"/>
+      <c r="H10" s="11"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1216,22 +1222,22 @@
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G11" s="6"/>
+      <c r="F11" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G11" s="7"/>
       <c r="H11" s="1"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
       <c r="L11" s="2"/>
       <c r="M11" s="2"/>
-      <c r="N11" s="6"/>
+      <c r="N11" s="7"/>
       <c r="O11" s="1"/>
       <c r="P11"/>
       <c r="Q11"/>
@@ -1251,10 +1257,10 @@
     </row>
     <row r="12" ht="14.25">
       <c r="A12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C12" s="2"/>
-      <c r="D12" s="6"/>
+      <c r="D12" s="7"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12"/>
@@ -1263,19 +1269,19 @@
       <c r="J12"/>
       <c r="K12"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="5" t="s">
-        <v>30</v>
+      <c r="M12" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="N12"/>
       <c r="O12" s="1"/>
       <c r="P12"/>
       <c r="Q12"/>
       <c r="R12"/>
-      <c r="S12" s="6"/>
+      <c r="S12" s="7"/>
       <c r="T12" s="2"/>
       <c r="U12"/>
-      <c r="V12" s="7" t="s">
-        <v>30</v>
+      <c r="V12" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="W12"/>
       <c r="X12"/>
@@ -1288,11 +1294,11 @@
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="6"/>
+      <c r="E13" s="7"/>
       <c r="F13" s="2"/>
       <c r="G13"/>
       <c r="H13" s="1"/>
@@ -1302,8 +1308,8 @@
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13"/>
-      <c r="O13" s="7" t="s">
-        <v>30</v>
+      <c r="O13" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="P13"/>
       <c r="Q13"/>
@@ -1314,7 +1320,7 @@
       <c r="V13" s="1"/>
       <c r="W13"/>
       <c r="X13"/>
-      <c r="Y13" s="6"/>
+      <c r="Y13" s="7"/>
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
       <c r="AB13"/>
@@ -1323,7 +1329,7 @@
     </row>
     <row r="14" s="3" customFormat="1" ht="14.25">
       <c r="A14" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -1333,29 +1339,29 @@
       <c r="G14" s="3"/>
       <c r="H14" s="4"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="8" t="s">
-        <v>44</v>
+      <c r="J14" s="9" t="s">
+        <v>45</v>
       </c>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="3"/>
-      <c r="O14" s="11"/>
+      <c r="O14" s="12"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
       <c r="U14" s="3"/>
-      <c r="V14" s="12" t="s">
-        <v>30</v>
+      <c r="V14" s="13" t="s">
+        <v>31</v>
       </c>
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
       <c r="Y14" s="3"/>
       <c r="Z14" s="3"/>
       <c r="AA14" s="3"/>
-      <c r="AB14" s="9"/>
+      <c r="AB14" s="10"/>
       <c r="AC14" s="4"/>
       <c r="AD14" s="3"/>
       <c r="AE14" s="3"/>
@@ -1369,14 +1375,14 @@
     </row>
     <row r="15" ht="14.25">
       <c r="A15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B15" s="6"/>
+        <v>46</v>
+      </c>
+      <c r="B15" s="7"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="6"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="1"/>
       <c r="I15"/>
       <c r="J15"/>
@@ -1403,7 +1409,7 @@
     </row>
     <row r="16" ht="14.25">
       <c r="A16" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -1411,8 +1417,8 @@
       <c r="F16" s="2"/>
       <c r="G16"/>
       <c r="H16" s="1"/>
-      <c r="I16" s="5" t="s">
-        <v>30</v>
+      <c r="I16" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="J16"/>
       <c r="K16"/>
@@ -1438,13 +1444,13 @@
     </row>
     <row r="17" ht="14.25">
       <c r="A17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
-      <c r="G17" s="6"/>
+      <c r="G17" s="7"/>
       <c r="H17" s="1"/>
       <c r="I17"/>
       <c r="J17"/>
@@ -1452,8 +1458,8 @@
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
       <c r="N17"/>
-      <c r="O17" s="7" t="s">
-        <v>30</v>
+      <c r="O17" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="P17"/>
       <c r="Q17"/>
@@ -1462,36 +1468,36 @@
       <c r="T17" s="2"/>
       <c r="U17"/>
       <c r="V17" s="1"/>
-      <c r="W17" s="6"/>
+      <c r="W17" s="7"/>
       <c r="X17"/>
       <c r="Y17"/>
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
       <c r="AB17"/>
-      <c r="AC17" s="7" t="s">
-        <v>30</v>
+      <c r="AC17" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="AD17" s="2"/>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="5" t="s">
-        <v>30</v>
+      <c r="G18" s="7"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="J18"/>
       <c r="K18"/>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
-      <c r="N18" s="6"/>
+      <c r="N18" s="7"/>
       <c r="O18" s="1"/>
       <c r="P18"/>
       <c r="Q18"/>
@@ -1511,7 +1517,7 @@
     </row>
     <row r="19" s="3" customFormat="1" ht="14.25">
       <c r="A19" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1526,17 +1532,17 @@
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
       <c r="N19" s="3"/>
-      <c r="O19" s="12" t="s">
-        <v>30</v>
+      <c r="O19" s="13" t="s">
+        <v>31</v>
       </c>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
-      <c r="S19" s="9"/>
+      <c r="S19" s="10"/>
       <c r="T19" s="3"/>
       <c r="U19" s="3"/>
-      <c r="V19" s="12" t="s">
-        <v>30</v>
+      <c r="V19" s="13" t="s">
+        <v>31</v>
       </c>
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
@@ -1557,13 +1563,13 @@
     </row>
     <row r="20" ht="14.25">
       <c r="A20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
-      <c r="F20" s="5" t="s">
-        <v>30</v>
+      <c r="F20" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="G20"/>
       <c r="H20" s="1"/>
@@ -1585,8 +1591,8 @@
       <c r="X20"/>
       <c r="Y20"/>
       <c r="Z20" s="2"/>
-      <c r="AA20" s="5" t="s">
-        <v>30</v>
+      <c r="AA20" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="AB20"/>
       <c r="AC20" s="1"/>
@@ -1594,7 +1600,7 @@
     </row>
     <row r="21" ht="14.25">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1618,20 +1624,20 @@
       <c r="V21" s="1"/>
       <c r="W21"/>
       <c r="X21"/>
-      <c r="Y21" s="5" t="s">
-        <v>30</v>
+      <c r="Y21" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="Z21" s="2"/>
       <c r="AA21" s="2"/>
       <c r="AB21"/>
-      <c r="AC21" s="7" t="s">
-        <v>30</v>
+      <c r="AC21" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="AD21" s="2"/>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1643,13 +1649,13 @@
       <c r="J22"/>
       <c r="K22"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="5" t="s">
-        <v>30</v>
+      <c r="M22" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="N22"/>
       <c r="O22" s="1"/>
-      <c r="P22" s="5" t="s">
-        <v>30</v>
+      <c r="P22" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="Q22"/>
       <c r="R22"/>
@@ -1668,13 +1674,13 @@
     </row>
     <row r="23" ht="14.25">
       <c r="A23" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>30</v>
+        <v>54</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>31</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>

</xml_diff>